<commit_message>
Rename preprocessing folder, updating gpt-example file and def get_prompt_messages
</commit_message>
<xml_diff>
--- a/data/describe/team_buildup.xlsx
+++ b/data/describe/team_buildup.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEA48A4A-48C8-4C34-A541-87D9E6E22053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henri\Desktop\Fotballanalyser\context_engineering_test\Context-Engineering-TWELVE-team-work\data\describe\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C1EBF6-DA78-4345-896D-D805E575F514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -49,21 +54,12 @@
     <t>What metrics do we use to evaluate a team's build-up?</t>
   </si>
   <si>
-    <t>We evaluate team build-up with Build-up Ending with Finish %, First-Line Break %, Second-Last-Line Break %, Turnover % in Build-up, Opponent Box Entries Within 7s After Turnover, Opponent Shot Probability Within 7s After Turnover. Together, these metrics describe how threatening, direct, progressive and secure a team's build-up is.</t>
-  </si>
-  <si>
     <t>general</t>
   </si>
   <si>
     <t>qa</t>
   </si>
   <si>
-    <t>What is team build-up?</t>
-  </si>
-  <si>
-    <t>Team build-up describes how a team starts and progresses possession before the attack becomes fully established. In this context, the focus is on how build-up creates threat, breaks lines, reaches finishes and how exposed the team becomes if it loses the ball.</t>
-  </si>
-  <si>
     <t>What does Build-up Ending with Finish % measure?</t>
   </si>
   <si>
@@ -341,13 +337,22 @@
   </si>
   <si>
     <t>Optional content type label. Set to 'qa' for all rows here.</t>
+  </si>
+  <si>
+    <t>What is a team build-up?</t>
+  </si>
+  <si>
+    <t>Team build-up describes how a team starts and progresses possession before the attack becomes fully established. In this analysis the build-up phase is starting when the ball is in the teams own third and the player in possession is under pressure. In this context, the focus is on how build-up creates threat, breaks lines, reaches finishes and how exposed the team becomes if it loses the ball.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We evaluate team build-up with Build-up Ending with Finish %, First-Line Break %, Turnover % in Build-up, Opponent Box Entries Within 7s After Turnover, Opponent Shot Probability Within 7s After Turnover. Together, these metrics describe how strong a team progress the ball forward towards goal, how secure they are in controlling the ball without losing the ball, and how good they are at avoiding opposition chances after turnovers. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -730,7 +735,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
     <col min="2" max="2" width="120" customWidth="1"/>
@@ -738,7 +743,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -752,592 +757,592 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="45.75">
+    <row r="2" spans="1:4" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C30" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="2" t="s">
+      <c r="B31" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C31" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C32" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C33" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="2" t="s">
+      <c r="B34" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="30.75">
-      <c r="A34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B35" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C35" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="30.75">
-      <c r="A35" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="30.75">
-      <c r="A36" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C37" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="30.75">
-      <c r="A37" s="2" t="s">
+      <c r="B38" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C38" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="30.75">
-      <c r="A38" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="30.75">
-      <c r="A39" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="30.75">
-      <c r="A40" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="30.75">
-      <c r="A41" s="2" t="s">
+      <c r="B42" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C42" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="30.75">
-      <c r="A42" s="2" t="s">
+      <c r="B43" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="30.75">
-      <c r="A43" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="C43" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1351,50 +1356,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated description file, describe and gpt-example file
</commit_message>
<xml_diff>
--- a/data/describe/team_buildup.xlsx
+++ b/data/describe/team_buildup.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henri\Desktop\Fotballanalyser\context_engineering_test\Context-Engineering-TWELVE-team-work\data\describe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C1EBF6-DA78-4345-896D-D805E575F514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F354D4-ED5E-471E-93E7-69573023FA6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="104">
   <si>
     <t>user</t>
   </si>
@@ -60,126 +60,30 @@
     <t>qa</t>
   </si>
   <si>
-    <t>What does Build-up Ending with Finish % measure?</t>
-  </si>
-  <si>
-    <t>Build-up Ending with Finish % measures How often a build-up sequence ends with a shot or other finish action.</t>
-  </si>
-  <si>
     <t>buildup_that_ends_with_finish_pct</t>
   </si>
   <si>
-    <t>What does a high value in Build-up Ending with Finish % mean?</t>
-  </si>
-  <si>
-    <t>A high value suggests the team converts build-up into shots regularly and can complete attacks once progression is established.</t>
-  </si>
-  <si>
-    <t>What does a low value in Build-up Ending with Finish % mean?</t>
-  </si>
-  <si>
-    <t>A low value suggests the team reaches fewer finishes from build-up and may struggle to turn control into actual shots.</t>
-  </si>
-  <si>
-    <t>How should I interpret Build-up Ending with Finish % in a team build-up context?</t>
-  </si>
-  <si>
-    <t>High values fit efficient attacking teams; low values fit teams that progress but fail to complete attacks. Read alongside build-up to create %. A team may create promising situations without finishing them often.</t>
-  </si>
-  <si>
-    <t>Is a higher or lower value better for Build-up Ending with Finish %?</t>
-  </si>
-  <si>
-    <t>Build-up Ending with Finish %: Higher is usually better. In this dataset the median is 26.36, upper-quartile is around 30.13, and top-end is around 33.34. The lowest example in the sample is Crystal Palace and the highest is Manchester City.</t>
-  </si>
-  <si>
-    <t>What does First-Line Break % measure?</t>
-  </si>
-  <si>
-    <t>First-Line Break % measures How often the team breaks the opponent’s first defensive line during build-up.</t>
-  </si>
-  <si>
     <t>first_line_break_pct_buildup</t>
   </si>
   <si>
-    <t>What does a high value in First-Line Break % mean?</t>
-  </si>
-  <si>
     <t>A high value suggests the team is comfortable escaping initial pressure and finding routes through the first wave of the press.</t>
   </si>
   <si>
-    <t>What does a low value in First-Line Break % mean?</t>
-  </si>
-  <si>
-    <t>A low value suggests the team can struggle to play through the first pressure line and may recycle or go long under stress.</t>
-  </si>
-  <si>
-    <t>How should I interpret First-Line Break % in a team build-up context?</t>
-  </si>
-  <si>
-    <t>High values fit press-resistant build-up; low values fit teams that are easier to slow down early in possession. This should be paired with turnover rate. Some teams break the first line often but take big risks to do it.</t>
-  </si>
-  <si>
-    <t>Is a higher or lower value better for First-Line Break %?</t>
-  </si>
-  <si>
-    <t>First-Line Break %: Higher is usually better. In this dataset the median is 27.43, upper-quartile is around 30.60, and top-end is around 32.15. The lowest example in the sample is Nottingham and the highest is Tottenham.</t>
-  </si>
-  <si>
-    <t>What does Second-Last-Line Break % measure?</t>
-  </si>
-  <si>
-    <t>Second-Last-Line Break % measures How often the team breaks into or through the deeper defensive line during build-up.</t>
-  </si>
-  <si>
     <t>second_last_line_break_pct_buildup</t>
   </si>
   <si>
-    <t>What does a high value in Second-Last-Line Break % mean?</t>
-  </si>
-  <si>
-    <t>A high value suggests the team can progress into advanced zones and threaten the defensive block with penetrative passing or carries.</t>
-  </si>
-  <si>
-    <t>What does a low value in Second-Last-Line Break % mean?</t>
-  </si>
-  <si>
-    <t>A low value suggests the team struggles to move possession into the most dangerous zones from build-up.</t>
-  </si>
-  <si>
-    <t>How should I interpret Second-Last-Line Break % in a team build-up context?</t>
-  </si>
-  <si>
-    <t>High values fit teams with advanced progression and penetration; low values fit teams that stay in front of the block too often. Read together with finish and create metrics. Penetration matters most when it also leads to threat.</t>
-  </si>
-  <si>
-    <t>Is a higher or lower value better for Second-Last-Line Break %?</t>
-  </si>
-  <si>
-    <t>Second-Last-Line Break %: Higher is usually better. In this dataset the median is 17.31, upper-quartile is around 18.85, and top-end is around 20.61. The lowest example in the sample is Nottingham and the highest is Chelsea.</t>
-  </si>
-  <si>
     <t>What does Turnover % in Build-up measure?</t>
   </si>
   <si>
-    <t>Turnover % in Build-up measures How often the team loses the ball during build-up.</t>
-  </si>
-  <si>
     <t>turnover_pct_buildup</t>
   </si>
   <si>
     <t>What does a high value in Turnover % in Build-up mean?</t>
   </si>
   <si>
-    <t>A high value suggests the team is loose or overly aggressive in possession and gives the ball away too often in early phases.</t>
-  </si>
-  <si>
     <t>What does a low value in Turnover % in Build-up mean?</t>
   </si>
   <si>
-    <t>A low value suggests the team is secure in build-up and protects possession well before attacks develop.</t>
-  </si>
-  <si>
     <t>How should I interpret Turnover % in Build-up in a team build-up context?</t>
   </si>
   <si>
@@ -192,54 +96,24 @@
     <t>Turnover % in Build-up: Lower is better. In this dataset the median is 9.48, upper-quartile is around 10.24, and top-end is around 11.33. The lowest example in the sample is Liverpool and the highest is Ipswich Town.</t>
   </si>
   <si>
-    <t>What does Opponent Box Entries Within 7s After Turnover measure?</t>
-  </si>
-  <si>
     <t>Opponent Box Entries Within 7s After Turnover measures How often the opponent reaches the box quickly after the team loses the ball in build-up.</t>
   </si>
   <si>
     <t>opp_box_entries_within_7s_after_turnover</t>
   </si>
   <si>
-    <t>What does a high value in Opponent Box Entries Within 7s After Turnover mean?</t>
-  </si>
-  <si>
-    <t>A high value suggests the team is vulnerable immediately after losing possession and can be attacked before it resets.</t>
-  </si>
-  <si>
-    <t>What does a low value in Opponent Box Entries Within 7s After Turnover mean?</t>
-  </si>
-  <si>
-    <t>A low value suggests the team limits immediate damage after turnovers, either through rest defence, spacing or counterpressure.</t>
-  </si>
-  <si>
-    <t>How should I interpret Opponent Box Entries Within 7s After Turnover in a team build-up context?</t>
-  </si>
-  <si>
-    <t>High values fit fragile rest-defence structures; low values fit teams that are better protected behind the ball. This is a consequence metric. It should be read together with turnover rate and the team’s overall build-up risk profile.</t>
-  </si>
-  <si>
-    <t>Is a higher or lower value better for Opponent Box Entries Within 7s After Turnover?</t>
-  </si>
-  <si>
     <t>Opponent Box Entries Within 7s After Turnover: Lower is better. In this dataset the median is 0.0835, upper-quartile is around 0.0998, and top-end is around 0.1340. The lowest example in the sample is Nottingham and the highest is Aston Villa.</t>
   </si>
   <si>
     <t>What does Opponent Shot Probability Within 7s After Turnover measure?</t>
   </si>
   <si>
-    <t>Opponent Shot Probability Within 7s After Turnover measures How likely the opponent is to get a shot quickly after a build-up turnover.</t>
-  </si>
-  <si>
     <t>opp_shot_probability_within_7s_after_turnover</t>
   </si>
   <si>
     <t>What does a high value in Opponent Shot Probability Within 7s After Turnover mean?</t>
   </si>
   <si>
-    <t>A high value suggests turnovers are especially costly, with losses often turning into high-value transitions against.</t>
-  </si>
-  <si>
     <t>What does a low value in Opponent Shot Probability Within 7s After Turnover mean?</t>
   </si>
   <si>
@@ -249,78 +123,15 @@
     <t>How should I interpret Opponent Shot Probability Within 7s After Turnover in a team build-up context?</t>
   </si>
   <si>
-    <t>High values fit open, vulnerable build-up; low values fit controlled build-up with stronger defensive protection. A team can be secure in pure turnover rate but still be badly exposed when a turnover does happen.</t>
-  </si>
-  <si>
     <t>Is a higher or lower value better for Opponent Shot Probability Within 7s After Turnover?</t>
   </si>
   <si>
     <t>Opponent Shot Probability Within 7s After Turnover: Lower is better. In this dataset the median is 0.1066, upper-quartile is around 0.1297, and top-end is around 0.1379. The lowest example in the sample is West Ham and the highest is Southampton.</t>
   </si>
   <si>
-    <t>What does the profile 'Penetrative progressor' mean?</t>
-  </si>
-  <si>
-    <t>This team is effective at moving the ball through multiple defensive layers. It does not just escape pressure; it carries or passes into advanced zones consistently.</t>
-  </si>
-  <si>
     <t>quality_profile</t>
   </si>
   <si>
-    <t>When would you describe a team as 'Penetrative progressor'?</t>
-  </si>
-  <si>
-    <t>This label fits when the team shows the following signal: High First-Line Break %, high Second-Last-Line Break %. Check whether the advanced progression actually leads to finish %.</t>
-  </si>
-  <si>
-    <t>What does the profile 'Safe but sterile build-up' mean?</t>
-  </si>
-  <si>
-    <t>This team can keep the ball without taking many risks, but the build-up lacks incision. Possession looks secure, though it does not consistently produce dangerous attacks.</t>
-  </si>
-  <si>
-    <t>When would you describe a team as 'Safe but sterile build-up'?</t>
-  </si>
-  <si>
-    <t>This label fits when the team shows the following signal: Low Turnover %, low Finish %. The team may need more tempo, more verticality or more penetration between lines.</t>
-  </si>
-  <si>
-    <t>What does the profile 'Risky creator' mean?</t>
-  </si>
-  <si>
-    <t>This team does create danger from build-up, but it pays a clear price for that ambition. The possession game is aggressive and productive, yet it can leave the team exposed when moves break down.</t>
-  </si>
-  <si>
-    <t>When would you describe a team as 'Risky creator'?</t>
-  </si>
-  <si>
-    <t>This label fits when the team shows the following signal: High high Turnover %, high post-turnover exposure. Balance the attacking upside against the defensive cost of turnovers.</t>
-  </si>
-  <si>
-    <t>What does the profile 'Fragile in rest defence' mean?</t>
-  </si>
-  <si>
-    <t>The problem is not only losing the ball; it is what happens next. When this team turns the ball over in build-up, the opponent can attack the box and generate shots quickly.</t>
-  </si>
-  <si>
-    <t>When would you describe a team as 'Fragile in rest defence'?</t>
-  </si>
-  <si>
-    <t>This label fits when the team shows the following signal: High Opponent Box Entries within 7s, high Opponent Shot Probability within 7s. Look at spacing, rest defence and immediate counterpressure around possession losses.</t>
-  </si>
-  <si>
-    <t>What does the profile 'Secure under pressure' mean?</t>
-  </si>
-  <si>
-    <t>This team looks composed in early possession phases. It can play through pressure without giving the ball away often, and it limits the damage if possession is lost.</t>
-  </si>
-  <si>
-    <t>When would you describe a team as 'Secure under pressure'?</t>
-  </si>
-  <si>
-    <t>This label fits when the team shows the following signal: Low Turnover %, low post-turnover exposure, decent line-break rates. Security is valuable, but check that the build-up also produces enough attacking payoff.</t>
-  </si>
-  <si>
     <t>field</t>
   </si>
   <si>
@@ -342,10 +153,202 @@
     <t>What is a team build-up?</t>
   </si>
   <si>
-    <t>Team build-up describes how a team starts and progresses possession before the attack becomes fully established. In this analysis the build-up phase is starting when the ball is in the teams own third and the player in possession is under pressure. In this context, the focus is on how build-up creates threat, breaks lines, reaches finishes and how exposed the team becomes if it loses the ball.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">We evaluate team build-up with Build-up Ending with Finish %, First-Line Break %, Turnover % in Build-up, Opponent Box Entries Within 7s After Turnover, Opponent Shot Probability Within 7s After Turnover. Together, these metrics describe how strong a team progress the ball forward towards goal, how secure they are in controlling the ball without losing the ball, and how good they are at avoiding opposition chances after turnovers. </t>
+    <t>This metric measure the share of teams build-ups that progress into midfield. A high value indicate the team is strong in controlling the ball and efficient in progressing the ball forward in build-up</t>
+  </si>
+  <si>
+    <t>quality profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We evaluate team build-up with first_line_break_pct_buildup, progression_to_midfield_pct, buildup_that_ends_with_finish_pct, turnover_pct_buildup, opp_box_entries_within_7s_after_turnover and opp_shot_probability_within_7s_after_turnover. Together, these metrics describe how efficient a team progress the ball forward, how secure they are in controlling the ball without losing it, and how good they are at avoiding opposition chances after turnovers. </t>
+  </si>
+  <si>
+    <t>Team build-up describes what happens when the team are having possession in their own third. In this context, the focus is on the ability to move the ball forward up the pitch, break opposition pressing lines, and how to stop opposition after a turnover if they lose the ball.</t>
+  </si>
+  <si>
+    <t>Buildup that ends with finish measures the share of build-ups that team manage to progress into an attacking, into a finish phase. A finish phase means the ball is either in final third, or in middle third with the defensive line close to their penalty area.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High values fit teams that are strong in progressing the ball from build-up, through midfield and into attack; low values fit teams fail to progress into attack. This is a metric for progression, it does not say anything about the number of shots for the team. </t>
+  </si>
+  <si>
+    <t>What does buildup that ends with finish pct measure?</t>
+  </si>
+  <si>
+    <t>What does a high value in buildup that ends with finish pct mean?</t>
+  </si>
+  <si>
+    <t>What does a low value in buildup that ends with finish pct measure?</t>
+  </si>
+  <si>
+    <t>How should I interpret buildup that ends with finish pct in a team build-up context?</t>
+  </si>
+  <si>
+    <t>Is a higher or lower value better for buildup that ends with finish pct?</t>
+  </si>
+  <si>
+    <t>buildup that ends with finish pct: Higher is better. In this dataset the lowest example in the sample is Crystal Palace and the highest is Manchester City.</t>
+  </si>
+  <si>
+    <t>first line break pct buildup measures how often the team breaks the opponent’s first defensive line during build-up.</t>
+  </si>
+  <si>
+    <t>What does a low value in first line break pct buildup mean?</t>
+  </si>
+  <si>
+    <t>A low value suggests the team can struggle to play through the first pressure line. They might recycle the ball more without breaking the first pressure or go long under stress. As the metric measure passes, teams might have also used carries to progresss thorugh the pressure.</t>
+  </si>
+  <si>
+    <t>High values fit press-resistant build-up; low values fit teams that take less risk in their build-up passing.  Some teams break the first line often but take big risks to do it. Effective teams which break lines often are making it difficult for the opposition to press high.</t>
+  </si>
+  <si>
+    <t>first line break pct: Higher is usually better. In this dataset the median is 27.43, upper-quartile is around 30.60, and top-end is around 32.15. The lowest example in the sample is Nottingham and the highest is Tottenham.</t>
+  </si>
+  <si>
+    <t>Turnover % in Build-up measures the share of team build-ups that ends with a turnover, where opponent win the ball.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A high value suggests the team is loose or overly aggressive in possession and gives the ball away too often in build-up. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A low value suggests the team is secure in build-up and protects possession well during progression in build-up. </t>
+  </si>
+  <si>
+    <t>A high value suggests the team is vulnerable immediately after losing possession in build-up, and team struggle to stop opponents from enter the the penalty area.</t>
+  </si>
+  <si>
+    <t>A low value suggests the team limits immediate damage after turnovers, either through quick recovery runs, counterpressure and ability to stop opponents from moving the ball into the box.</t>
+  </si>
+  <si>
+    <t>High values fit teams which loose the ball in dangerous positions during build-up, and teams which struggle to recover after the turnover. Low values fit teams that are better protected behind the ball, which loose the ball in less dangerous positions, and recover better when the turnover happens. This is a consequence metric. It should be read together with turnover rate and the team’s overall build-up play.</t>
+  </si>
+  <si>
+    <t>A high value suggests turnovers are especially costly for the team, with losses often turning into high-value transitions against.</t>
+  </si>
+  <si>
+    <t>Opponent Shot Probability Within 7s After Turnover measures How likely the opponent is to get a shot quickly after a build-up turnover. The metric measure the average probability for a shot within 7 sec from the turnover.</t>
+  </si>
+  <si>
+    <t>High values fit loss in possession at a bad place, allowing opposition in good shooting positions, indicating a high risk, and less controlled build-up; low values fit controlled build-up with stronger defensive protection. A team can be secure in pure turnover rate but still be badly exposed when a turnover does happen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How would you describe a team that are very strong controlling  the ball in build-up? </t>
+  </si>
+  <si>
+    <t>A team which is strong in controlling the ball could be described strong in recycling the ball, and often manage to play thas strong in progression_to_midfield_pct, turnover_pct_buildup, "first_line_break_pct_buildup</t>
+  </si>
+  <si>
+    <t>What does  progression to midfield pct  means?</t>
+  </si>
+  <si>
+    <t>What does a low value in  progression to midfield pct  means?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> progression to midfield pct measure the teams ability to keep the possession and progress the ball into midfield. The turnover measure the share of build-ups that ends in turnover. </t>
+  </si>
+  <si>
+    <t>What does build-ups that break the first defensive line of pressure measure?</t>
+  </si>
+  <si>
+    <t>What does a high value in build-ups that break the first defensive line of pressure mean?</t>
+  </si>
+  <si>
+    <t>How should I interpret build-ups that break the first defensive line of pressure in a build-up context?</t>
+  </si>
+  <si>
+    <t>Is a higher or lower value better for build-ups that break the first defensive line of pressure?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A low value tells the team is struggling to control, and progress the ball in build-up. A low value is also a clear sign of build-ups that ends in turnovers and chaotic phases without stable progression. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A low value suggests the team less often manage to progress the ball into attack. This tells they lack the ability to keep the ball during progression from the team, and possession is disturbed by the opposition.  </t>
+  </si>
+  <si>
+    <t>A high value tells the team manage to move the ball forward with control, consistently. It give the team a good foundation for creatin chances in the later stage.It also indicates a team which might be able to break the high press, when the opponent press high.</t>
+  </si>
+  <si>
+    <t>What are the difference between  progression to midfield pct  and turnovers?</t>
+  </si>
+  <si>
+    <t>Which metric/datapoints are most important for build-up?</t>
+  </si>
+  <si>
+    <t>How well they progress the ball into attacking zones (buildup that ends with finish pct) and the ability to avoid turnovers (turnovers during build-up) are two of the most important metrics when evaluating teams build-up play.</t>
+  </si>
+  <si>
+    <t>How would you describe a team which is good or outstanding in terms of Turnover % in Build-up?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team that manage to control the ball during build-up and rarely loose the ball. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">How would you describe a team which is good or outstanding in terms of Turnover % in Build-up, but below average or poor in terms of Opponent Box Entries Within 7s After Turnover and Opponent Shot Probability Within 7s After Turnover? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team which is strong on the ball during build-up, but concede chances after loosing the ball. This tell they often loose the ball in dangerous areas which leads to box entries and shot from the opponent. </t>
+  </si>
+  <si>
+    <t>What does it imply if a team is a good or excellent in terms of progression to midfield pct, and average, below average og poor in build-ups that progress into a finish phase?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This tells the team is very efficient when playing out from the back, and easyli get into midfield, but struggle to get into the final third. </t>
+  </si>
+  <si>
+    <t>If you want to know about team player you can select your prefered team in the bar to the left!</t>
+  </si>
+  <si>
+    <t>I want to know about another team?</t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in nearly all metrics?</t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in terms of build-ups that progress into a finish phase?</t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in terms of build-ups that break the first defensive line of pressure?</t>
+  </si>
+  <si>
+    <t>A team which is good or excellent in terms of build-ups that progress into a finish phase manage to play out from the back, break through the opponent pressure and progress through the middle third into attack. These teams can have different style of play, but they are all strong in progressing the ball into the final third.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team which is good or excellent in terms of build-ups that break the first defensive line of pressure are agressive in trying to play thorugh the first line of pressure from the opponent. Such passes can be highly effective, and break the opposition press and allow further progression forward.  However, these passes can also lead to dangerous turnovers, so this metric should not be interpreted in isolation. </t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in terms of turnovers during build-up?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team which is good or excellent in terms of turnovers during build-up are controlled in possession in their own third, and try to progress forward with control and rarely takes high risk during build-up. </t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in terms of opposition box entries shortly after turnovers?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team which is good or excellent in terms of opposition box entries shortly after turnovers are having a great balance between control and risk during build-up, which   contribute to less situations where opponents move into the box after turnovers. </t>
+  </si>
+  <si>
+    <t>A team which is good or excellent in terms of opposition shot probability shortly after turnovers are playing with a a great balance between control and risk during build-up, which contribute to less shooting opportunities for the opponent after turnovers. Such teams manage to be in a position to avoid good shooting opportunities when the turnovers happens.</t>
+  </si>
+  <si>
+    <t>What does a high value in opposition box entries shortly after turnovers mean?</t>
+  </si>
+  <si>
+    <t>What does a low value in opposition box entries shortly after turnovers mean?</t>
+  </si>
+  <si>
+    <t>How should I interpret opposition box entries shortly after turnovers in a team build-up context?</t>
+  </si>
+  <si>
+    <t>Is a higher or lower value better for opposition box entries shortly after turnovers?</t>
+  </si>
+  <si>
+    <t>What does Opponent opposition box entries shortly after turnovers measure?</t>
+  </si>
+  <si>
+    <t>What does it imply if a team is good or excellent in terms of opposition shot probability?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A team which is good or excellent in nearly all metrics is brilliant in progressing the ball forward with controlled possession, and rarely loose the ball in dangerous areas during build-up, which results in less opposition chances from turnovers. </t>
   </si>
 </sst>
 </file>
@@ -426,8 +429,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EmbedReadyDescribe" displayName="EmbedReadyDescribe" ref="A1:D43">
-  <autoFilter ref="A1:D43" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EmbedReadyDescribe" displayName="EmbedReadyDescribe" ref="A1:D60">
+  <autoFilter ref="A1:D60" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="user"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="assistant"/>
@@ -734,10 +737,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="60" customWidth="1"/>
+    <col min="1" max="1" width="94.81640625" customWidth="1"/>
     <col min="2" max="2" width="120" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
@@ -762,7 +765,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
@@ -771,12 +774,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>100</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>5</v>
@@ -787,13 +790,13 @@
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>6</v>
@@ -801,13 +804,13 @@
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>6</v>
@@ -815,13 +818,13 @@
     </row>
     <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>6</v>
@@ -829,13 +832,13 @@
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>6</v>
@@ -843,13 +846,13 @@
     </row>
     <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>6</v>
@@ -857,13 +860,13 @@
     </row>
     <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>6</v>
@@ -871,13 +874,13 @@
     </row>
     <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>6</v>
@@ -885,13 +888,13 @@
     </row>
     <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>6</v>
@@ -899,13 +902,13 @@
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>6</v>
@@ -913,13 +916,13 @@
     </row>
     <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>6</v>
@@ -927,13 +930,13 @@
     </row>
     <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>6</v>
@@ -941,13 +944,13 @@
     </row>
     <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>6</v>
@@ -955,13 +958,13 @@
     </row>
     <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>6</v>
@@ -969,13 +972,13 @@
     </row>
     <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>6</v>
@@ -983,69 +986,69 @@
     </row>
     <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>6</v>
@@ -1053,13 +1056,13 @@
     </row>
     <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>6</v>
@@ -1067,13 +1070,13 @@
     </row>
     <row r="24" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>6</v>
@@ -1081,13 +1084,13 @@
     </row>
     <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>6</v>
@@ -1095,27 +1098,27 @@
     </row>
     <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>6</v>
@@ -1123,225 +1126,233 @@
     </row>
     <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>63</v>
+      <c r="A29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" t="s">
+        <v>38</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="B31" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="C32" s="2" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>72</v>
+      <c r="A33" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" t="s">
+        <v>78</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>74</v>
+    <row r="34" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>77</v>
+    <row r="35" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>79</v>
+    <row r="36" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" t="s">
+        <v>84</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>81</v>
+    <row r="37" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" t="s">
+        <v>103</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>83</v>
+    <row r="38" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" t="s">
+        <v>90</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B39" s="2" t="s">
+    <row r="39" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>89</v>
+      </c>
+      <c r="B39" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" t="s">
+        <v>93</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" t="s">
+        <v>95</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>86</v>
+      </c>
+      <c r="B43" t="s">
         <v>85</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="C43" s="2" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D43" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C44" t="s">
+        <v>39</v>
+      </c>
+      <c r="D44" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1364,10 +1375,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -1375,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>96</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1383,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1391,7 +1402,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>98</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -1399,7 +1410,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>99</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Style analyst: Add team build up style analysis
</commit_message>
<xml_diff>
--- a/data/describe/team_buildup.xlsx
+++ b/data/describe/team_buildup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henri\Desktop\Fotballanalyser\context_engineering_test\Context-Engineering-TWELVE-team-work\data\describe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johulf\Context-Engineering-TWELVE-team-work\data\describe\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{C6811CFA-6828-4BF1-9E2F-F3BD3F1032BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30630" yWindow="1200" windowWidth="21600" windowHeight="12585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -355,7 +355,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -748,7 +748,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="74.42578125" style="4" customWidth="1"/>
     <col min="2" max="2" width="120" style="4" customWidth="1"/>
@@ -756,7 +756,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -770,7 +770,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60.75">
+    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -784,7 +784,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30.75">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -798,7 +798,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="30.75">
+    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -812,7 +812,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="30.75">
+    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -826,7 +826,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="30.75">
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -840,7 +840,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="30.75">
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30.75">
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -868,7 +868,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="30.75">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -882,7 +882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="30.75">
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -896,7 +896,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="45.75">
+    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -910,7 +910,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="30.75">
+    <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
@@ -924,7 +924,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30.75">
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -938,7 +938,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="30.75">
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -952,7 +952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="30.75">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -966,7 +966,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="30.75">
+    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
@@ -980,7 +980,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="30.75">
+    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -994,7 +994,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="30.75">
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="30.75">
+    <row r="19" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>43</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="30.75">
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="30.75">
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>48</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="45.75">
+    <row r="22" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="30.75">
+    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="45.75">
+    <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="45.75">
+    <row r="25" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>57</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="45.75">
+    <row r="26" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>59</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="45.75">
+    <row r="27" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>61</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="45.75">
+    <row r="28" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>63</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="45.75">
+    <row r="29" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>65</v>
       </c>
@@ -1162,7 +1162,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="45.75">
+    <row r="30" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>68</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="45.75">
+    <row r="31" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>70</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="45.75">
+    <row r="32" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>72</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="45.75">
+    <row r="33" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>74</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="43.5" customHeight="1">
+    <row r="34" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>76</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="43.5" customHeight="1">
+    <row r="35" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>79</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="43.5" customHeight="1">
+    <row r="36" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>81</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="43.5" customHeight="1">
+    <row r="37" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>83</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="43.5" customHeight="1">
+    <row r="38" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>85</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="43.5" customHeight="1">
+    <row r="39" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>87</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="43.5" customHeight="1">
+    <row r="40" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>89</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="43.5" customHeight="1">
+    <row r="41" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>91</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="43.5" customHeight="1">
+    <row r="42" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>93</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="43.5" customHeight="1">
+    <row r="43" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>95</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C44" t="s">
         <v>97</v>
       </c>
@@ -1377,13 +1377,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>98</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>

</xml_diff>